<commit_message>
implement changes according to 20260720 Software tool test results 04-05-26
</commit_message>
<xml_diff>
--- a/assets/program_logic_v7.xlsx
+++ b/assets/program_logic_v7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7100f48b682a1df6/Work/20251027 IEC TC86 Digital Tool/repo/standards-tool/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E79C11-43BB-49F6-898B-1BB2A8DB6806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{00E79C11-43BB-49F6-898B-1BB2A8DB6806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{058B6A23-B264-47A4-A005-B5EF375C2140}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="8" xr2:uid="{0D1380F2-B44E-49CB-9379-F623B51E2EAA}"/>
   </bookViews>
@@ -28,6 +28,9 @@
     <sheet name="Filter 5" sheetId="20" r:id="rId13"/>
     <sheet name="INFO" sheetId="21" r:id="rId14"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Filter 1'!$A$1:$C$28</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -49,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="188">
   <si>
     <t>Connector type</t>
   </si>
@@ -671,6 +674,24 @@
   </si>
   <si>
     <t>IEC 61753-022-13</t>
+  </si>
+  <si>
+    <t>Note 4</t>
+  </si>
+  <si>
+    <t>IEC PAS</t>
+  </si>
+  <si>
+    <t>IEC TR</t>
+  </si>
+  <si>
+    <t>IEC</t>
+  </si>
+  <si>
+    <t>ISO/IEC</t>
+  </si>
+  <si>
+    <t>For automatic linking to work, standards must start with one of the following prefixes - all other prefixes will fail or produce unexpected results:</t>
   </si>
 </sst>
 </file>
@@ -2488,7 +2509,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0B3FE3C-7D18-4B18-A8AC-ABE63533F11D}">
-  <dimension ref="A2:C82"/>
+  <dimension ref="A2:C88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="31"/>
@@ -2911,14 +2932,42 @@
         <v>165</v>
       </c>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B81" s="31" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B82" s="31" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="B84" s="33" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B85" s="31" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B86" s="31" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B87" s="31" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B88" s="31" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -4516,6 +4565,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C28" xr:uid="{D2B2682D-C6CB-4DE7-9E39-FE9FD68A45F6}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>